<commit_message>
Update RSI screener report 2026-09-12 08:02 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -466,438 +466,514 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>IRFC</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>264.1</v>
+        <v>81.09</v>
       </c>
       <c r="C2" t="n">
-        <v>28.04</v>
+        <v>27.12</v>
       </c>
       <c r="D2" t="n">
-        <v>30.95</v>
+        <v>38.35</v>
       </c>
       <c r="E2" t="n">
-        <v>-37.36</v>
+        <v>-39.32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>878</v>
+        <v>1927</v>
       </c>
       <c r="C3" t="n">
-        <v>28.82</v>
+        <v>27.7</v>
       </c>
       <c r="D3" t="n">
-        <v>38.59</v>
+        <v>36.96</v>
       </c>
       <c r="E3" t="n">
-        <v>-30.68</v>
+        <v>-26.51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IRFC</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>83.40000000000001</v>
+        <v>865</v>
       </c>
       <c r="C4" t="n">
-        <v>29.29</v>
+        <v>27.84</v>
       </c>
       <c r="D4" t="n">
-        <v>39.1</v>
+        <v>38.11</v>
       </c>
       <c r="E4" t="n">
-        <v>-37.59</v>
+        <v>-31.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1973.4</v>
+        <v>991</v>
       </c>
       <c r="C5" t="n">
-        <v>30.43</v>
+        <v>30.05</v>
       </c>
       <c r="D5" t="n">
-        <v>38.25</v>
+        <v>44.63</v>
       </c>
       <c r="E5" t="n">
-        <v>-26</v>
+        <v>-22.03</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>712.1</v>
+        <v>167.4</v>
       </c>
       <c r="C6" t="n">
-        <v>31.47</v>
+        <v>30.53</v>
       </c>
       <c r="D6" t="n">
-        <v>37.68</v>
+        <v>35.52</v>
       </c>
       <c r="E6" t="n">
-        <v>-29.46</v>
+        <v>-38.61</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1010</v>
+        <v>708.25</v>
       </c>
       <c r="C7" t="n">
-        <v>32.29</v>
+        <v>30.87</v>
       </c>
       <c r="D7" t="n">
-        <v>45.79</v>
+        <v>37.27</v>
       </c>
       <c r="E7" t="n">
-        <v>-20.54</v>
+        <v>-29.84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>407.6</v>
+        <v>391.85</v>
       </c>
       <c r="C8" t="n">
-        <v>32.73</v>
+        <v>31.25</v>
       </c>
       <c r="D8" t="n">
-        <v>44.1</v>
+        <v>35.73</v>
       </c>
       <c r="E8" t="n">
-        <v>-25.08</v>
+        <v>-33.76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMBUJACEM</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>405</v>
+        <v>5009</v>
       </c>
       <c r="C9" t="n">
-        <v>34.59</v>
+        <v>32.97</v>
       </c>
       <c r="D9" t="n">
-        <v>37.35</v>
+        <v>44.5</v>
       </c>
       <c r="E9" t="n">
-        <v>-31.54</v>
+        <v>-20.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>355.6</v>
+        <v>5009</v>
       </c>
       <c r="C10" t="n">
-        <v>34.76</v>
+        <v>32.97</v>
       </c>
       <c r="D10" t="n">
-        <v>46.08</v>
+        <v>44.5</v>
       </c>
       <c r="E10" t="n">
-        <v>-26.13</v>
+        <v>-20.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>272.1</v>
+        <v>530</v>
       </c>
       <c r="C11" t="n">
-        <v>34.76</v>
+        <v>33.52</v>
       </c>
       <c r="D11" t="n">
-        <v>40.2</v>
+        <v>35.25</v>
       </c>
       <c r="E11" t="n">
-        <v>-65.45</v>
+        <v>-32.72</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>176.4</v>
+        <v>263.7</v>
       </c>
       <c r="C12" t="n">
-        <v>35.37</v>
+        <v>33.88</v>
       </c>
       <c r="D12" t="n">
-        <v>37.2</v>
+        <v>39.75</v>
       </c>
       <c r="E12" t="n">
-        <v>-35.31</v>
+        <v>-66.51000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>311.5</v>
+        <v>22785</v>
       </c>
       <c r="C13" t="n">
-        <v>36.23</v>
+        <v>33.89</v>
       </c>
       <c r="D13" t="n">
-        <v>34.96</v>
+        <v>38.93</v>
       </c>
       <c r="E13" t="n">
-        <v>-56.71</v>
+        <v>-24.08</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5130</v>
+        <v>301.1</v>
       </c>
       <c r="C14" t="n">
-        <v>36.27</v>
+        <v>33.94</v>
       </c>
       <c r="D14" t="n">
-        <v>46.07</v>
+        <v>34.3</v>
       </c>
       <c r="E14" t="n">
-        <v>-18.58</v>
+        <v>-58.13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5130</v>
+        <v>353.45</v>
       </c>
       <c r="C15" t="n">
-        <v>36.27</v>
+        <v>34.29</v>
       </c>
       <c r="D15" t="n">
-        <v>46.07</v>
+        <v>45.8</v>
       </c>
       <c r="E15" t="n">
-        <v>-18.58</v>
+        <v>-26.58</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>VBL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>546.4</v>
+        <v>416.5</v>
       </c>
       <c r="C16" t="n">
-        <v>36.71</v>
+        <v>36.23</v>
       </c>
       <c r="D16" t="n">
-        <v>36.89</v>
+        <v>45.02</v>
       </c>
       <c r="E16" t="n">
-        <v>-30.64</v>
+        <v>-23.44</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>239</v>
+        <v>313.8</v>
       </c>
       <c r="C17" t="n">
-        <v>37.32</v>
+        <v>36.34</v>
       </c>
       <c r="D17" t="n">
-        <v>47</v>
+        <v>42.62</v>
       </c>
       <c r="E17" t="n">
-        <v>-26.34</v>
+        <v>-18.85</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>332.5</v>
+        <v>1037.7</v>
       </c>
       <c r="C18" t="n">
-        <v>37.37</v>
+        <v>36.82</v>
       </c>
       <c r="D18" t="n">
-        <v>48.44</v>
+        <v>34.35</v>
       </c>
       <c r="E18" t="n">
-        <v>-18.94</v>
+        <v>-38.59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>266</v>
+        <v>238.13</v>
       </c>
       <c r="C19" t="n">
-        <v>37.72</v>
+        <v>36.93</v>
       </c>
       <c r="D19" t="n">
-        <v>46.78</v>
+        <v>46.79</v>
       </c>
       <c r="E19" t="n">
-        <v>-17.11</v>
+        <v>-26.61</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>318.7</v>
+        <v>333.4</v>
       </c>
       <c r="C20" t="n">
-        <v>37.79</v>
+        <v>38.02</v>
       </c>
       <c r="D20" t="n">
-        <v>43.2</v>
+        <v>48.65</v>
       </c>
       <c r="E20" t="n">
-        <v>-17.58</v>
+        <v>-18.72</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12694</v>
+        <v>232.5</v>
       </c>
       <c r="C21" t="n">
-        <v>39.01</v>
+        <v>38.11</v>
       </c>
       <c r="D21" t="n">
-        <v>47.62</v>
+        <v>46.15</v>
       </c>
       <c r="E21" t="n">
-        <v>-26.59</v>
+        <v>-22.86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>23855</v>
+        <v>12590</v>
       </c>
       <c r="C22" t="n">
-        <v>39.06</v>
+        <v>38.17</v>
       </c>
       <c r="D22" t="n">
-        <v>42.43</v>
+        <v>47.16</v>
       </c>
       <c r="E22" t="n">
-        <v>-21.75</v>
+        <v>-27.19</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>MUTHOOTFIN</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>234.65</v>
+        <v>2792.1</v>
       </c>
       <c r="C23" t="n">
-        <v>39.17</v>
+        <v>38.3</v>
       </c>
       <c r="D23" t="n">
-        <v>46.74</v>
+        <v>51.01</v>
       </c>
       <c r="E23" t="n">
-        <v>-22.15</v>
+        <v>-31.76</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1155</v>
+        <v>1700.6</v>
       </c>
       <c r="C24" t="n">
-        <v>39.38</v>
+        <v>38.94</v>
       </c>
       <c r="D24" t="n">
-        <v>45.48</v>
+        <v>48.28</v>
       </c>
       <c r="E24" t="n">
-        <v>-16.04</v>
+        <v>-19.39</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3690</v>
+      </c>
+      <c r="C25" t="n">
+        <v>39.11</v>
+      </c>
+      <c r="D25" t="n">
+        <v>45</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-22.73</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2200.8</v>
+      </c>
+      <c r="C26" t="n">
+        <v>39.41</v>
+      </c>
+      <c r="D26" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-33.81</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C27" t="n">
+        <v>39.62</v>
+      </c>
+      <c r="D27" t="n">
+        <v>48.38</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-15.72</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1257.5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="D28" t="n">
+        <v>43.74</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-21.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-09-19 08:11 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,73 +470,73 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81.09</v>
+        <v>81.5</v>
       </c>
       <c r="C2" t="n">
-        <v>27.12</v>
+        <v>28.13</v>
       </c>
       <c r="D2" t="n">
-        <v>38.35</v>
+        <v>38.48</v>
       </c>
       <c r="E2" t="n">
-        <v>-39.32</v>
+        <v>-39.02</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1927</v>
+        <v>262.3</v>
       </c>
       <c r="C3" t="n">
-        <v>27.7</v>
+        <v>28.93</v>
       </c>
       <c r="D3" t="n">
-        <v>36.96</v>
+        <v>30.44</v>
       </c>
       <c r="E3" t="n">
-        <v>-26.51</v>
+        <v>-37.78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>865</v>
+        <v>383.25</v>
       </c>
       <c r="C4" t="n">
-        <v>27.84</v>
+        <v>29.25</v>
       </c>
       <c r="D4" t="n">
-        <v>38.11</v>
+        <v>34.91</v>
       </c>
       <c r="E4" t="n">
-        <v>-31.7</v>
+        <v>-35.22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>991</v>
+        <v>1942.2</v>
       </c>
       <c r="C5" t="n">
-        <v>30.05</v>
+        <v>29.92</v>
       </c>
       <c r="D5" t="n">
-        <v>44.63</v>
+        <v>37.34</v>
       </c>
       <c r="E5" t="n">
-        <v>-22.03</v>
+        <v>-25.41</v>
       </c>
     </row>
     <row r="6">
@@ -546,73 +546,73 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>167.4</v>
+        <v>166.83</v>
       </c>
       <c r="C6" t="n">
-        <v>30.53</v>
+        <v>30.24</v>
       </c>
       <c r="D6" t="n">
-        <v>35.52</v>
+        <v>35.42</v>
       </c>
       <c r="E6" t="n">
-        <v>-38.61</v>
+        <v>-38.82</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>708.25</v>
+        <v>880</v>
       </c>
       <c r="C7" t="n">
-        <v>30.87</v>
+        <v>30.77</v>
       </c>
       <c r="D7" t="n">
-        <v>37.27</v>
+        <v>38.67</v>
       </c>
       <c r="E7" t="n">
-        <v>-29.84</v>
+        <v>-29.82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMBUJACEM</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>391.85</v>
+        <v>342.55</v>
       </c>
       <c r="C8" t="n">
-        <v>31.25</v>
+        <v>31.95</v>
       </c>
       <c r="D8" t="n">
-        <v>35.73</v>
+        <v>44.33</v>
       </c>
       <c r="E8" t="n">
-        <v>-33.76</v>
+        <v>-28.84</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5009</v>
+        <v>22600</v>
       </c>
       <c r="C9" t="n">
-        <v>32.97</v>
+        <v>33.27</v>
       </c>
       <c r="D9" t="n">
-        <v>44.5</v>
+        <v>38.48</v>
       </c>
       <c r="E9" t="n">
-        <v>-20.5</v>
+        <v>-24.69</v>
       </c>
     </row>
     <row r="10">
@@ -622,358 +622,320 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5009</v>
+        <v>4998</v>
       </c>
       <c r="C10" t="n">
-        <v>32.97</v>
+        <v>33.72</v>
       </c>
       <c r="D10" t="n">
-        <v>44.5</v>
+        <v>44.36</v>
       </c>
       <c r="E10" t="n">
-        <v>-20.5</v>
+        <v>-19.19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>530</v>
+        <v>4998</v>
       </c>
       <c r="C11" t="n">
-        <v>33.52</v>
+        <v>33.72</v>
       </c>
       <c r="D11" t="n">
-        <v>35.25</v>
+        <v>44.36</v>
       </c>
       <c r="E11" t="n">
-        <v>-32.72</v>
+        <v>-19.19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>263.7</v>
+        <v>323.65</v>
       </c>
       <c r="C12" t="n">
-        <v>33.88</v>
+        <v>33.9</v>
       </c>
       <c r="D12" t="n">
-        <v>39.75</v>
+        <v>46.41</v>
       </c>
       <c r="E12" t="n">
-        <v>-66.51000000000001</v>
+        <v>-21.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>22785</v>
+        <v>12103</v>
       </c>
       <c r="C13" t="n">
-        <v>33.89</v>
+        <v>34.51</v>
       </c>
       <c r="D13" t="n">
-        <v>38.93</v>
+        <v>45.13</v>
       </c>
       <c r="E13" t="n">
-        <v>-24.08</v>
+        <v>-30.01</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>301.1</v>
+        <v>267.6</v>
       </c>
       <c r="C14" t="n">
-        <v>33.94</v>
+        <v>34.7</v>
       </c>
       <c r="D14" t="n">
-        <v>34.3</v>
+        <v>39.96</v>
       </c>
       <c r="E14" t="n">
-        <v>-58.13</v>
+        <v>-66.02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>353.45</v>
+        <v>303.8</v>
       </c>
       <c r="C15" t="n">
-        <v>34.29</v>
+        <v>35.09</v>
       </c>
       <c r="D15" t="n">
-        <v>45.8</v>
+        <v>34.44</v>
       </c>
       <c r="E15" t="n">
-        <v>-26.58</v>
+        <v>-57.71</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>416.5</v>
+        <v>234.94</v>
       </c>
       <c r="C16" t="n">
-        <v>36.23</v>
+        <v>35.45</v>
       </c>
       <c r="D16" t="n">
-        <v>45.02</v>
+        <v>46.06</v>
       </c>
       <c r="E16" t="n">
-        <v>-23.44</v>
+        <v>-27.59</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>313.8</v>
+        <v>2105</v>
       </c>
       <c r="C17" t="n">
-        <v>36.34</v>
+        <v>35.6</v>
       </c>
       <c r="D17" t="n">
-        <v>42.62</v>
+        <v>33.66</v>
       </c>
       <c r="E17" t="n">
-        <v>-18.85</v>
+        <v>-36.69</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1037.7</v>
+        <v>1013.7</v>
       </c>
       <c r="C18" t="n">
-        <v>36.82</v>
+        <v>35.77</v>
       </c>
       <c r="D18" t="n">
-        <v>34.35</v>
+        <v>46.02</v>
       </c>
       <c r="E18" t="n">
-        <v>-38.59</v>
+        <v>-20.24</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>238.13</v>
+        <v>312</v>
       </c>
       <c r="C19" t="n">
-        <v>36.93</v>
+        <v>35.82</v>
       </c>
       <c r="D19" t="n">
-        <v>46.79</v>
+        <v>42.42</v>
       </c>
       <c r="E19" t="n">
-        <v>-26.61</v>
+        <v>-19.32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>333.4</v>
+        <v>1226.4</v>
       </c>
       <c r="C20" t="n">
-        <v>38.02</v>
+        <v>36.9</v>
       </c>
       <c r="D20" t="n">
-        <v>48.65</v>
+        <v>42.09</v>
       </c>
       <c r="E20" t="n">
-        <v>-18.72</v>
+        <v>-22.98</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>MUTHOOTFIN</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>232.5</v>
+        <v>2771.4</v>
       </c>
       <c r="C21" t="n">
-        <v>38.11</v>
+        <v>37.75</v>
       </c>
       <c r="D21" t="n">
-        <v>46.15</v>
+        <v>50.59</v>
       </c>
       <c r="E21" t="n">
-        <v>-22.86</v>
+        <v>-32.27</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>12590</v>
+        <v>731</v>
       </c>
       <c r="C22" t="n">
-        <v>38.17</v>
+        <v>38.33</v>
       </c>
       <c r="D22" t="n">
-        <v>47.16</v>
+        <v>39.8</v>
       </c>
       <c r="E22" t="n">
-        <v>-27.19</v>
+        <v>-27.59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MUTHOOTFIN</t>
+          <t>VBL</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2792.1</v>
+        <v>421.95</v>
       </c>
       <c r="C23" t="n">
-        <v>38.3</v>
+        <v>38.35</v>
       </c>
       <c r="D23" t="n">
-        <v>51.01</v>
+        <v>45.56</v>
       </c>
       <c r="E23" t="n">
-        <v>-31.76</v>
+        <v>-22.44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1700.6</v>
+        <v>232.8</v>
       </c>
       <c r="C24" t="n">
-        <v>38.94</v>
+        <v>38.36</v>
       </c>
       <c r="D24" t="n">
-        <v>48.28</v>
+        <v>46.23</v>
       </c>
       <c r="E24" t="n">
-        <v>-19.39</v>
+        <v>-22.76</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DMART</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3690</v>
+        <v>1051.4</v>
       </c>
       <c r="C25" t="n">
-        <v>39.11</v>
+        <v>38.37</v>
       </c>
       <c r="D25" t="n">
-        <v>45</v>
+        <v>34.75</v>
       </c>
       <c r="E25" t="n">
-        <v>-22.73</v>
+        <v>-37.78</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2200.8</v>
+        <v>11014</v>
       </c>
       <c r="C26" t="n">
-        <v>39.41</v>
+        <v>39.9</v>
       </c>
       <c r="D26" t="n">
-        <v>34.88</v>
+        <v>48.47</v>
       </c>
       <c r="E26" t="n">
-        <v>-33.81</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>ULTRACEMCO</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>11000</v>
-      </c>
-      <c r="C27" t="n">
-        <v>39.62</v>
-      </c>
-      <c r="D27" t="n">
-        <v>48.38</v>
-      </c>
-      <c r="E27" t="n">
-        <v>-15.72</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>RELIANCE</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1257.5</v>
-      </c>
-      <c r="C28" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="D28" t="n">
-        <v>43.74</v>
-      </c>
-      <c r="E28" t="n">
-        <v>-21.03</v>
+        <v>-15.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-09-26 08:44 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -470,35 +470,35 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81.5</v>
+        <v>79.95</v>
       </c>
       <c r="C2" t="n">
-        <v>28.13</v>
+        <v>26.62</v>
       </c>
       <c r="D2" t="n">
-        <v>38.48</v>
+        <v>37.99</v>
       </c>
       <c r="E2" t="n">
-        <v>-39.02</v>
+        <v>-40.18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>262.3</v>
+        <v>164.02</v>
       </c>
       <c r="C3" t="n">
-        <v>28.93</v>
+        <v>28.83</v>
       </c>
       <c r="D3" t="n">
-        <v>30.44</v>
+        <v>34.92</v>
       </c>
       <c r="E3" t="n">
-        <v>-37.78</v>
+        <v>-39.85</v>
       </c>
     </row>
     <row r="4">
@@ -508,54 +508,54 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>383.25</v>
+        <v>383.8</v>
       </c>
       <c r="C4" t="n">
-        <v>29.25</v>
+        <v>29.3</v>
       </c>
       <c r="D4" t="n">
-        <v>34.91</v>
+        <v>34.96</v>
       </c>
       <c r="E4" t="n">
-        <v>-35.22</v>
+        <v>-33.76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1942.2</v>
+        <v>983.2</v>
       </c>
       <c r="C5" t="n">
-        <v>29.92</v>
+        <v>29.82</v>
       </c>
       <c r="D5" t="n">
-        <v>37.34</v>
+        <v>44.17</v>
       </c>
       <c r="E5" t="n">
-        <v>-25.41</v>
+        <v>-22.64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>166.83</v>
+        <v>1942.9</v>
       </c>
       <c r="C6" t="n">
-        <v>30.24</v>
+        <v>30.14</v>
       </c>
       <c r="D6" t="n">
-        <v>35.42</v>
+        <v>37.36</v>
       </c>
       <c r="E6" t="n">
-        <v>-38.82</v>
+        <v>-25.38</v>
       </c>
     </row>
     <row r="7">
@@ -584,35 +584,35 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>342.55</v>
+        <v>338</v>
       </c>
       <c r="C8" t="n">
-        <v>31.95</v>
+        <v>31</v>
       </c>
       <c r="D8" t="n">
-        <v>44.33</v>
+        <v>43.7</v>
       </c>
       <c r="E8" t="n">
-        <v>-28.84</v>
+        <v>-29.79</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22600</v>
+        <v>4937.5</v>
       </c>
       <c r="C9" t="n">
-        <v>33.27</v>
+        <v>32.11</v>
       </c>
       <c r="D9" t="n">
-        <v>38.48</v>
+        <v>43.62</v>
       </c>
       <c r="E9" t="n">
-        <v>-24.69</v>
+        <v>-20.17</v>
       </c>
     </row>
     <row r="10">
@@ -622,54 +622,54 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4998</v>
+        <v>4937.5</v>
       </c>
       <c r="C10" t="n">
-        <v>33.72</v>
+        <v>32.11</v>
       </c>
       <c r="D10" t="n">
-        <v>44.36</v>
+        <v>43.62</v>
       </c>
       <c r="E10" t="n">
-        <v>-19.19</v>
+        <v>-20.17</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4998</v>
+        <v>290.45</v>
       </c>
       <c r="C11" t="n">
-        <v>33.72</v>
+        <v>32.12</v>
       </c>
       <c r="D11" t="n">
-        <v>44.36</v>
+        <v>33.77</v>
       </c>
       <c r="E11" t="n">
-        <v>-19.19</v>
+        <v>-59.57</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>323.65</v>
+        <v>22520</v>
       </c>
       <c r="C12" t="n">
-        <v>33.9</v>
+        <v>32.9</v>
       </c>
       <c r="D12" t="n">
-        <v>46.41</v>
+        <v>38.29</v>
       </c>
       <c r="E12" t="n">
-        <v>-21.1</v>
+        <v>-24.96</v>
       </c>
     </row>
     <row r="13">
@@ -679,16 +679,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>12103</v>
+        <v>12065</v>
       </c>
       <c r="C13" t="n">
-        <v>34.51</v>
+        <v>34.23</v>
       </c>
       <c r="D13" t="n">
-        <v>45.13</v>
+        <v>44.97</v>
       </c>
       <c r="E13" t="n">
-        <v>-30.01</v>
+        <v>-30.23</v>
       </c>
     </row>
     <row r="14">
@@ -698,244 +698,244 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>267.6</v>
+        <v>266.35</v>
       </c>
       <c r="C14" t="n">
-        <v>34.7</v>
+        <v>34.56</v>
       </c>
       <c r="D14" t="n">
-        <v>39.96</v>
+        <v>39.89</v>
       </c>
       <c r="E14" t="n">
-        <v>-66.02</v>
+        <v>-66.18000000000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>303.8</v>
+        <v>2082</v>
       </c>
       <c r="C15" t="n">
-        <v>35.09</v>
+        <v>34.73</v>
       </c>
       <c r="D15" t="n">
-        <v>34.44</v>
+        <v>33.38</v>
       </c>
       <c r="E15" t="n">
-        <v>-57.71</v>
+        <v>-37.38</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>234.94</v>
+        <v>1000.2</v>
       </c>
       <c r="C16" t="n">
-        <v>35.45</v>
+        <v>34.93</v>
       </c>
       <c r="D16" t="n">
-        <v>46.06</v>
+        <v>33.3</v>
       </c>
       <c r="E16" t="n">
-        <v>-27.59</v>
+        <v>-40.81</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2105</v>
+        <v>269</v>
       </c>
       <c r="C17" t="n">
-        <v>35.6</v>
+        <v>35.26</v>
       </c>
       <c r="D17" t="n">
-        <v>33.66</v>
+        <v>32.31</v>
       </c>
       <c r="E17" t="n">
-        <v>-36.69</v>
+        <v>-36.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1013.7</v>
+        <v>235.26</v>
       </c>
       <c r="C18" t="n">
-        <v>35.77</v>
+        <v>35.73</v>
       </c>
       <c r="D18" t="n">
-        <v>46.02</v>
+        <v>46.13</v>
       </c>
       <c r="E18" t="n">
-        <v>-20.24</v>
+        <v>-27.49</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>312</v>
+        <v>326.6</v>
       </c>
       <c r="C19" t="n">
-        <v>35.82</v>
+        <v>36.15</v>
       </c>
       <c r="D19" t="n">
-        <v>42.42</v>
+        <v>47.04</v>
       </c>
       <c r="E19" t="n">
-        <v>-19.32</v>
+        <v>-20.38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1226.4</v>
+        <v>312.95</v>
       </c>
       <c r="C20" t="n">
-        <v>36.9</v>
+        <v>36.36</v>
       </c>
       <c r="D20" t="n">
-        <v>42.09</v>
+        <v>42.52</v>
       </c>
       <c r="E20" t="n">
-        <v>-22.98</v>
+        <v>-18.83</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MUTHOOTFIN</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2771.4</v>
+        <v>531</v>
       </c>
       <c r="C21" t="n">
-        <v>37.75</v>
+        <v>36.61</v>
       </c>
       <c r="D21" t="n">
-        <v>50.59</v>
+        <v>35.34</v>
       </c>
       <c r="E21" t="n">
-        <v>-32.27</v>
+        <v>-32.58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>731</v>
+        <v>1226</v>
       </c>
       <c r="C22" t="n">
-        <v>38.33</v>
+        <v>36.86</v>
       </c>
       <c r="D22" t="n">
-        <v>39.8</v>
+        <v>42.07</v>
       </c>
       <c r="E22" t="n">
-        <v>-27.59</v>
+        <v>-23</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>MAZDOCK</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>421.95</v>
+        <v>2199.6</v>
       </c>
       <c r="C23" t="n">
-        <v>38.35</v>
+        <v>38.14</v>
       </c>
       <c r="D23" t="n">
-        <v>45.56</v>
+        <v>48.55</v>
       </c>
       <c r="E23" t="n">
-        <v>-22.44</v>
+        <v>-24.78</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>232.8</v>
+        <v>2669.3</v>
       </c>
       <c r="C24" t="n">
-        <v>38.36</v>
+        <v>39.15</v>
       </c>
       <c r="D24" t="n">
-        <v>46.23</v>
+        <v>39.89</v>
       </c>
       <c r="E24" t="n">
-        <v>-22.76</v>
+        <v>-44.76</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1051.4</v>
+        <v>735.6</v>
       </c>
       <c r="C25" t="n">
-        <v>38.37</v>
+        <v>39.75</v>
       </c>
       <c r="D25" t="n">
-        <v>34.75</v>
+        <v>40.29</v>
       </c>
       <c r="E25" t="n">
-        <v>-37.78</v>
+        <v>-27.13</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>11014</v>
+        <v>2444</v>
       </c>
       <c r="C26" t="n">
-        <v>39.9</v>
+        <v>39.88</v>
       </c>
       <c r="D26" t="n">
-        <v>48.47</v>
+        <v>46.43</v>
       </c>
       <c r="E26" t="n">
-        <v>-15.61</v>
+        <v>-17.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-10-03 09:18 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,35 +470,35 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79.95</v>
+        <v>77.06</v>
       </c>
       <c r="C2" t="n">
-        <v>26.62</v>
+        <v>24.02</v>
       </c>
       <c r="D2" t="n">
-        <v>37.99</v>
+        <v>37.07</v>
       </c>
       <c r="E2" t="n">
-        <v>-40.18</v>
+        <v>-42.34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>164.02</v>
+        <v>1836</v>
       </c>
       <c r="C3" t="n">
-        <v>28.83</v>
+        <v>24.13</v>
       </c>
       <c r="D3" t="n">
-        <v>34.92</v>
+        <v>34.77</v>
       </c>
       <c r="E3" t="n">
-        <v>-39.85</v>
+        <v>-29.48</v>
       </c>
     </row>
     <row r="4">
@@ -508,92 +508,92 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>383.8</v>
+        <v>362.25</v>
       </c>
       <c r="C4" t="n">
-        <v>29.3</v>
+        <v>24.71</v>
       </c>
       <c r="D4" t="n">
-        <v>34.96</v>
+        <v>32.97</v>
       </c>
       <c r="E4" t="n">
-        <v>-33.76</v>
+        <v>-37.24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>983.2</v>
+        <v>159.35</v>
       </c>
       <c r="C5" t="n">
-        <v>29.82</v>
+        <v>26.59</v>
       </c>
       <c r="D5" t="n">
-        <v>44.17</v>
+        <v>34.29</v>
       </c>
       <c r="E5" t="n">
-        <v>-22.64</v>
+        <v>-41.56</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1942.9</v>
+        <v>957</v>
       </c>
       <c r="C6" t="n">
-        <v>30.14</v>
+        <v>26.84</v>
       </c>
       <c r="D6" t="n">
-        <v>37.36</v>
+        <v>42.87</v>
       </c>
       <c r="E6" t="n">
-        <v>-25.38</v>
+        <v>-24.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>880</v>
+        <v>318</v>
       </c>
       <c r="C7" t="n">
-        <v>30.77</v>
+        <v>27.18</v>
       </c>
       <c r="D7" t="n">
-        <v>38.67</v>
+        <v>41.48</v>
       </c>
       <c r="E7" t="n">
-        <v>-29.82</v>
+        <v>-33.94</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>338</v>
+        <v>840</v>
       </c>
       <c r="C8" t="n">
-        <v>31</v>
+        <v>27.34</v>
       </c>
       <c r="D8" t="n">
-        <v>43.7</v>
+        <v>37.18</v>
       </c>
       <c r="E8" t="n">
-        <v>-29.79</v>
+        <v>-33.01</v>
       </c>
     </row>
     <row r="9">
@@ -603,16 +603,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4937.5</v>
+        <v>4778</v>
       </c>
       <c r="C9" t="n">
-        <v>32.11</v>
+        <v>28.26</v>
       </c>
       <c r="D9" t="n">
-        <v>43.62</v>
+        <v>41.74</v>
       </c>
       <c r="E9" t="n">
-        <v>-20.17</v>
+        <v>-22.75</v>
       </c>
     </row>
     <row r="10">
@@ -622,260 +622,260 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4937.5</v>
+        <v>4778</v>
       </c>
       <c r="C10" t="n">
-        <v>32.11</v>
+        <v>28.26</v>
       </c>
       <c r="D10" t="n">
-        <v>43.62</v>
+        <v>41.74</v>
       </c>
       <c r="E10" t="n">
-        <v>-20.17</v>
+        <v>-22.75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>290.45</v>
+        <v>287.75</v>
       </c>
       <c r="C11" t="n">
-        <v>32.12</v>
+        <v>29.28</v>
       </c>
       <c r="D11" t="n">
-        <v>33.77</v>
+        <v>39.72</v>
       </c>
       <c r="E11" t="n">
-        <v>-59.57</v>
+        <v>-25.37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22520</v>
+        <v>11386</v>
       </c>
       <c r="C12" t="n">
-        <v>32.9</v>
+        <v>29.56</v>
       </c>
       <c r="D12" t="n">
-        <v>38.29</v>
+        <v>42.27</v>
       </c>
       <c r="E12" t="n">
-        <v>-24.96</v>
+        <v>-34.15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>12065</v>
+        <v>279.4</v>
       </c>
       <c r="C13" t="n">
-        <v>34.23</v>
+        <v>29.87</v>
       </c>
       <c r="D13" t="n">
-        <v>44.97</v>
+        <v>33.22</v>
       </c>
       <c r="E13" t="n">
-        <v>-30.23</v>
+        <v>-61.11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>266.35</v>
+        <v>21900</v>
       </c>
       <c r="C14" t="n">
-        <v>34.56</v>
+        <v>30.13</v>
       </c>
       <c r="D14" t="n">
-        <v>39.89</v>
+        <v>36.79</v>
       </c>
       <c r="E14" t="n">
-        <v>-66.18000000000001</v>
+        <v>-27.02</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2082</v>
+        <v>315.1</v>
       </c>
       <c r="C15" t="n">
-        <v>34.73</v>
+        <v>31.62</v>
       </c>
       <c r="D15" t="n">
-        <v>33.38</v>
+        <v>44.54</v>
       </c>
       <c r="E15" t="n">
-        <v>-37.38</v>
+        <v>-23.18</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1000.2</v>
+        <v>1167.7</v>
       </c>
       <c r="C16" t="n">
-        <v>34.93</v>
+        <v>31.69</v>
       </c>
       <c r="D16" t="n">
-        <v>33.3</v>
+        <v>39.23</v>
       </c>
       <c r="E16" t="n">
-        <v>-40.81</v>
+        <v>-26.67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>269</v>
+        <v>254.55</v>
       </c>
       <c r="C17" t="n">
-        <v>35.26</v>
+        <v>32.81</v>
       </c>
       <c r="D17" t="n">
-        <v>32.31</v>
+        <v>44.01</v>
       </c>
       <c r="E17" t="n">
-        <v>-36.2</v>
+        <v>-20.68</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>235.26</v>
+        <v>252.05</v>
       </c>
       <c r="C18" t="n">
-        <v>35.73</v>
+        <v>32.82</v>
       </c>
       <c r="D18" t="n">
-        <v>46.13</v>
+        <v>39.12</v>
       </c>
       <c r="E18" t="n">
-        <v>-27.49</v>
+        <v>-67.98999999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>326.6</v>
+        <v>230.82</v>
       </c>
       <c r="C19" t="n">
-        <v>36.15</v>
+        <v>33.58</v>
       </c>
       <c r="D19" t="n">
-        <v>47.04</v>
+        <v>45.17</v>
       </c>
       <c r="E19" t="n">
-        <v>-20.38</v>
+        <v>-28.86</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>MAZDOCK</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>312.95</v>
+        <v>2064</v>
       </c>
       <c r="C20" t="n">
-        <v>36.36</v>
+        <v>33.7</v>
       </c>
       <c r="D20" t="n">
-        <v>42.52</v>
+        <v>46.43</v>
       </c>
       <c r="E20" t="n">
-        <v>-18.83</v>
+        <v>-28.55</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>531</v>
+        <v>222.37</v>
       </c>
       <c r="C21" t="n">
-        <v>36.61</v>
+        <v>34.1</v>
       </c>
       <c r="D21" t="n">
-        <v>35.34</v>
+        <v>43.77</v>
       </c>
       <c r="E21" t="n">
-        <v>-32.58</v>
+        <v>-26.22</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1226</v>
+        <v>2075</v>
       </c>
       <c r="C22" t="n">
-        <v>36.86</v>
+        <v>34.46</v>
       </c>
       <c r="D22" t="n">
-        <v>42.07</v>
+        <v>33.63</v>
       </c>
       <c r="E22" t="n">
-        <v>-23</v>
+        <v>-37.59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MAZDOCK</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2199.6</v>
+        <v>2860</v>
       </c>
       <c r="C23" t="n">
-        <v>38.14</v>
+        <v>35.03</v>
       </c>
       <c r="D23" t="n">
-        <v>48.55</v>
+        <v>47.63</v>
       </c>
       <c r="E23" t="n">
         <v>-24.78</v>
@@ -884,58 +884,381 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2669.3</v>
+        <v>118.36</v>
       </c>
       <c r="C24" t="n">
-        <v>39.15</v>
+        <v>36.23</v>
       </c>
       <c r="D24" t="n">
-        <v>39.89</v>
+        <v>49.94</v>
       </c>
       <c r="E24" t="n">
-        <v>-44.76</v>
+        <v>-25.53</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>MUTHOOTFIN</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>735.6</v>
+        <v>2697.1</v>
       </c>
       <c r="C25" t="n">
-        <v>39.75</v>
+        <v>36.25</v>
       </c>
       <c r="D25" t="n">
-        <v>40.29</v>
+        <v>49.08</v>
       </c>
       <c r="E25" t="n">
-        <v>-27.13</v>
+        <v>-34.08</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2580</v>
+      </c>
+      <c r="C26" t="n">
+        <v>36.66</v>
+      </c>
+      <c r="D26" t="n">
+        <v>39.25</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-46.61</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>10710</v>
+      </c>
+      <c r="C27" t="n">
+        <v>36.77</v>
+      </c>
+      <c r="D27" t="n">
+        <v>46.37</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-17.94</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>721.2</v>
+      </c>
+      <c r="C28" t="n">
+        <v>36.89</v>
+      </c>
+      <c r="D28" t="n">
+        <v>38.84</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-28.56</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>534.2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>37.67</v>
+      </c>
+      <c r="D29" t="n">
+        <v>36.61</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-32.17</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>ASIANPAINT</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>2444</v>
-      </c>
-      <c r="C26" t="n">
-        <v>39.88</v>
-      </c>
-      <c r="D26" t="n">
-        <v>46.43</v>
-      </c>
-      <c r="E26" t="n">
-        <v>-17.67</v>
+      <c r="B30" t="n">
+        <v>2407</v>
+      </c>
+      <c r="C30" t="n">
+        <v>37.76</v>
+      </c>
+      <c r="D30" t="n">
+        <v>45.71</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-18.92</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1741.1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>38.24</v>
+      </c>
+      <c r="D31" t="n">
+        <v>50.21</v>
+      </c>
+      <c r="E31" t="n">
+        <v>-19.49</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>350.15</v>
+      </c>
+      <c r="C32" t="n">
+        <v>38.25</v>
+      </c>
+      <c r="D32" t="n">
+        <v>45.63</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-24.18</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>131.34</v>
+      </c>
+      <c r="C33" t="n">
+        <v>38.29</v>
+      </c>
+      <c r="D33" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-29.94</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1732.6</v>
+      </c>
+      <c r="C34" t="n">
+        <v>38.84</v>
+      </c>
+      <c r="D34" t="n">
+        <v>46.26</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-20.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>6920</v>
+      </c>
+      <c r="C35" t="n">
+        <v>38.85</v>
+      </c>
+      <c r="D35" t="n">
+        <v>55.67</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-15.51</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>954.1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>38.89</v>
+      </c>
+      <c r="D36" t="n">
+        <v>52.94</v>
+      </c>
+      <c r="E36" t="n">
+        <v>-22.29</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1035</v>
+      </c>
+      <c r="C37" t="n">
+        <v>38.94</v>
+      </c>
+      <c r="D37" t="n">
+        <v>35.44</v>
+      </c>
+      <c r="E37" t="n">
+        <v>-38.75</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>383.1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="D38" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-18.22</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1307.7</v>
+      </c>
+      <c r="C39" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="D39" t="n">
+        <v>51.56</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-15.08</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3693.4</v>
+      </c>
+      <c r="C40" t="n">
+        <v>39.29</v>
+      </c>
+      <c r="D40" t="n">
+        <v>49.73</v>
+      </c>
+      <c r="E40" t="n">
+        <v>-16.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2308.1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>39.37</v>
+      </c>
+      <c r="D41" t="n">
+        <v>48.64</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-20.46</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C42" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="D42" t="n">
+        <v>51.77</v>
+      </c>
+      <c r="E42" t="n">
+        <v>-18.56</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>178</v>
+      </c>
+      <c r="C43" t="n">
+        <v>39.96</v>
+      </c>
+      <c r="D43" t="n">
+        <v>52.04</v>
+      </c>
+      <c r="E43" t="n">
+        <v>-19.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-10-10 10:01 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,795 +470,890 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77.06</v>
+        <v>74.7</v>
       </c>
       <c r="C2" t="n">
-        <v>24.02</v>
+        <v>22.13</v>
       </c>
       <c r="D2" t="n">
-        <v>37.07</v>
+        <v>36.34</v>
       </c>
       <c r="E2" t="n">
-        <v>-42.34</v>
+        <v>-44.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1836</v>
+        <v>351.5</v>
       </c>
       <c r="C3" t="n">
-        <v>24.13</v>
+        <v>22.79</v>
       </c>
       <c r="D3" t="n">
-        <v>34.77</v>
+        <v>32.03</v>
       </c>
       <c r="E3" t="n">
-        <v>-29.48</v>
+        <v>-39.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AMBUJACEM</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>362.25</v>
+        <v>955</v>
       </c>
       <c r="C4" t="n">
-        <v>24.71</v>
+        <v>26.62</v>
       </c>
       <c r="D4" t="n">
-        <v>32.97</v>
+        <v>42.71</v>
       </c>
       <c r="E4" t="n">
-        <v>-37.24</v>
+        <v>-24.86</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>159.35</v>
+        <v>1856.7</v>
       </c>
       <c r="C5" t="n">
-        <v>26.59</v>
+        <v>27.16</v>
       </c>
       <c r="D5" t="n">
-        <v>34.29</v>
+        <v>35.27</v>
       </c>
       <c r="E5" t="n">
-        <v>-41.56</v>
+        <v>-28.69</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>957</v>
+        <v>11420</v>
       </c>
       <c r="C6" t="n">
-        <v>26.84</v>
+        <v>30.08</v>
       </c>
       <c r="D6" t="n">
-        <v>42.87</v>
+        <v>42.4</v>
       </c>
       <c r="E6" t="n">
-        <v>-24.7</v>
+        <v>-33.96</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>318</v>
+        <v>279.9</v>
       </c>
       <c r="C7" t="n">
-        <v>27.18</v>
+        <v>30.11</v>
       </c>
       <c r="D7" t="n">
-        <v>41.48</v>
+        <v>33.24</v>
       </c>
       <c r="E7" t="n">
-        <v>-33.94</v>
+        <v>-58.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>840</v>
+        <v>249.15</v>
       </c>
       <c r="C8" t="n">
-        <v>27.34</v>
+        <v>30.47</v>
       </c>
       <c r="D8" t="n">
-        <v>37.18</v>
+        <v>42.81</v>
       </c>
       <c r="E8" t="n">
-        <v>-33.01</v>
+        <v>-22.36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4778</v>
+        <v>312</v>
       </c>
       <c r="C9" t="n">
-        <v>28.26</v>
+        <v>30.51</v>
       </c>
       <c r="D9" t="n">
-        <v>41.74</v>
+        <v>43.9</v>
       </c>
       <c r="E9" t="n">
-        <v>-22.75</v>
+        <v>-23.94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4778</v>
+        <v>162.57</v>
       </c>
       <c r="C10" t="n">
-        <v>28.26</v>
+        <v>30.58</v>
       </c>
       <c r="D10" t="n">
-        <v>41.74</v>
+        <v>35.36</v>
       </c>
       <c r="E10" t="n">
-        <v>-22.75</v>
+        <v>-40.38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>287.75</v>
+        <v>4825</v>
       </c>
       <c r="C11" t="n">
-        <v>29.28</v>
+        <v>30.89</v>
       </c>
       <c r="D11" t="n">
-        <v>39.72</v>
+        <v>42.3</v>
       </c>
       <c r="E11" t="n">
-        <v>-25.37</v>
+        <v>-21.99</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11386</v>
+        <v>4825</v>
       </c>
       <c r="C12" t="n">
-        <v>29.56</v>
+        <v>30.89</v>
       </c>
       <c r="D12" t="n">
-        <v>42.27</v>
+        <v>42.3</v>
       </c>
       <c r="E12" t="n">
-        <v>-34.15</v>
+        <v>-21.99</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>279.4</v>
+        <v>860.5</v>
       </c>
       <c r="C13" t="n">
-        <v>29.87</v>
+        <v>31.55</v>
       </c>
       <c r="D13" t="n">
-        <v>33.22</v>
+        <v>38.23</v>
       </c>
       <c r="E13" t="n">
-        <v>-61.11</v>
+        <v>-31.38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>21900</v>
+        <v>327.8</v>
       </c>
       <c r="C14" t="n">
-        <v>30.13</v>
+        <v>31.63</v>
       </c>
       <c r="D14" t="n">
-        <v>36.79</v>
+        <v>42.65</v>
       </c>
       <c r="E14" t="n">
-        <v>-27.02</v>
+        <v>-31.91</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>315.1</v>
+        <v>22080</v>
       </c>
       <c r="C15" t="n">
-        <v>31.62</v>
+        <v>31.92</v>
       </c>
       <c r="D15" t="n">
-        <v>44.54</v>
+        <v>37.22</v>
       </c>
       <c r="E15" t="n">
-        <v>-23.18</v>
+        <v>-26.42</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>MAZDOCK</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1167.7</v>
+        <v>2010</v>
       </c>
       <c r="C16" t="n">
-        <v>31.69</v>
+        <v>32.11</v>
       </c>
       <c r="D16" t="n">
-        <v>39.23</v>
+        <v>45.6</v>
       </c>
       <c r="E16" t="n">
-        <v>-26.67</v>
+        <v>-30.42</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>254.55</v>
+        <v>1170.3</v>
       </c>
       <c r="C17" t="n">
-        <v>32.81</v>
+        <v>32.14</v>
       </c>
       <c r="D17" t="n">
-        <v>44.01</v>
+        <v>39.35</v>
       </c>
       <c r="E17" t="n">
-        <v>-20.68</v>
+        <v>-26.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>252.05</v>
+        <v>2796.2</v>
       </c>
       <c r="C18" t="n">
-        <v>32.82</v>
+        <v>33.14</v>
       </c>
       <c r="D18" t="n">
-        <v>39.12</v>
+        <v>46.33</v>
       </c>
       <c r="E18" t="n">
-        <v>-67.98999999999999</v>
+        <v>-26.46</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>230.82</v>
+        <v>221.27</v>
       </c>
       <c r="C19" t="n">
-        <v>33.58</v>
+        <v>33.6</v>
       </c>
       <c r="D19" t="n">
-        <v>45.17</v>
+        <v>43.51</v>
       </c>
       <c r="E19" t="n">
-        <v>-28.86</v>
+        <v>-26.59</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAZDOCK</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2064</v>
+        <v>2339.1</v>
       </c>
       <c r="C20" t="n">
-        <v>33.7</v>
+        <v>34.18</v>
       </c>
       <c r="D20" t="n">
-        <v>46.43</v>
+        <v>44.29</v>
       </c>
       <c r="E20" t="n">
-        <v>-28.55</v>
+        <v>-21.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>IOC</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>222.37</v>
+        <v>126.35</v>
       </c>
       <c r="C21" t="n">
-        <v>34.1</v>
+        <v>34.22</v>
       </c>
       <c r="D21" t="n">
-        <v>43.77</v>
+        <v>43.45</v>
       </c>
       <c r="E21" t="n">
-        <v>-26.22</v>
+        <v>-32.6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2075</v>
+        <v>707.25</v>
       </c>
       <c r="C22" t="n">
-        <v>34.46</v>
+        <v>34.32</v>
       </c>
       <c r="D22" t="n">
-        <v>33.63</v>
+        <v>37.19</v>
       </c>
       <c r="E22" t="n">
-        <v>-37.59</v>
+        <v>-29.94</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>MUTHOOTFIN</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2860</v>
+        <v>2624.7</v>
       </c>
       <c r="C23" t="n">
-        <v>35.03</v>
+        <v>34.35</v>
       </c>
       <c r="D23" t="n">
-        <v>47.63</v>
+        <v>47.66</v>
       </c>
       <c r="E23" t="n">
-        <v>-24.78</v>
+        <v>-35.85</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>118.36</v>
+        <v>368.15</v>
       </c>
       <c r="C24" t="n">
-        <v>36.23</v>
+        <v>34.58</v>
       </c>
       <c r="D24" t="n">
-        <v>49.94</v>
+        <v>51.66</v>
       </c>
       <c r="E24" t="n">
-        <v>-25.53</v>
+        <v>-21.41</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MUTHOOTFIN</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2697.1</v>
+        <v>264</v>
       </c>
       <c r="C25" t="n">
-        <v>36.25</v>
+        <v>35.72</v>
       </c>
       <c r="D25" t="n">
-        <v>49.08</v>
+        <v>39.93</v>
       </c>
       <c r="E25" t="n">
-        <v>-34.08</v>
+        <v>-66.48</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2580</v>
+        <v>300</v>
       </c>
       <c r="C26" t="n">
-        <v>36.66</v>
+        <v>35.82</v>
       </c>
       <c r="D26" t="n">
-        <v>39.25</v>
+        <v>41.14</v>
       </c>
       <c r="E26" t="n">
-        <v>-46.61</v>
+        <v>-22.19</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>10710</v>
+        <v>342.15</v>
       </c>
       <c r="C27" t="n">
-        <v>36.77</v>
+        <v>36.01</v>
       </c>
       <c r="D27" t="n">
-        <v>46.37</v>
+        <v>44.37</v>
       </c>
       <c r="E27" t="n">
-        <v>-17.94</v>
+        <v>-25.91</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>DMART</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>721.2</v>
+        <v>3516.8</v>
       </c>
       <c r="C28" t="n">
-        <v>36.89</v>
+        <v>36.03</v>
       </c>
       <c r="D28" t="n">
-        <v>38.84</v>
+        <v>42.84</v>
       </c>
       <c r="E28" t="n">
-        <v>-28.56</v>
+        <v>-24.02</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>534.2</v>
+        <v>10675</v>
       </c>
       <c r="C29" t="n">
-        <v>37.67</v>
+        <v>36.33</v>
       </c>
       <c r="D29" t="n">
-        <v>36.61</v>
+        <v>46.14</v>
       </c>
       <c r="E29" t="n">
-        <v>-32.17</v>
+        <v>-18.21</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2407</v>
+        <v>173.8</v>
       </c>
       <c r="C30" t="n">
-        <v>37.76</v>
+        <v>37.22</v>
       </c>
       <c r="D30" t="n">
-        <v>45.71</v>
+        <v>50.49</v>
       </c>
       <c r="E30" t="n">
-        <v>-18.92</v>
+        <v>-21.4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1741.1</v>
+        <v>1301</v>
       </c>
       <c r="C31" t="n">
-        <v>38.24</v>
+        <v>37.63</v>
       </c>
       <c r="D31" t="n">
-        <v>50.21</v>
+        <v>43.87</v>
       </c>
       <c r="E31" t="n">
-        <v>-19.49</v>
+        <v>-21.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>HDFCAMC</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>350.15</v>
+        <v>2262.5</v>
       </c>
       <c r="C32" t="n">
-        <v>38.25</v>
+        <v>37.82</v>
       </c>
       <c r="D32" t="n">
-        <v>45.63</v>
+        <v>47.37</v>
       </c>
       <c r="E32" t="n">
-        <v>-24.18</v>
+        <v>-22.03</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>131.34</v>
+        <v>266</v>
       </c>
       <c r="C33" t="n">
-        <v>38.29</v>
+        <v>37.84</v>
       </c>
       <c r="D33" t="n">
-        <v>45.3</v>
+        <v>31.56</v>
       </c>
       <c r="E33" t="n">
-        <v>-29.94</v>
+        <v>-36.91</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1732.6</v>
+        <v>861.65</v>
       </c>
       <c r="C34" t="n">
-        <v>38.84</v>
+        <v>38.04</v>
       </c>
       <c r="D34" t="n">
-        <v>46.26</v>
+        <v>44.47</v>
       </c>
       <c r="E34" t="n">
-        <v>-20.4</v>
+        <v>-19.42</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6920</v>
+        <v>235.8</v>
       </c>
       <c r="C35" t="n">
-        <v>38.85</v>
+        <v>38.08</v>
       </c>
       <c r="D35" t="n">
-        <v>55.67</v>
+        <v>46.54</v>
       </c>
       <c r="E35" t="n">
-        <v>-15.51</v>
+        <v>-27.32</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>954.1</v>
+        <v>1023.4</v>
       </c>
       <c r="C36" t="n">
-        <v>38.89</v>
+        <v>38.1</v>
       </c>
       <c r="D36" t="n">
-        <v>52.94</v>
+        <v>34.81</v>
       </c>
       <c r="E36" t="n">
-        <v>-22.29</v>
+        <v>-39.44</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1035</v>
+        <v>119.59</v>
       </c>
       <c r="C37" t="n">
-        <v>38.94</v>
+        <v>38.16</v>
       </c>
       <c r="D37" t="n">
-        <v>35.44</v>
+        <v>50.54</v>
       </c>
       <c r="E37" t="n">
-        <v>-38.75</v>
+        <v>-24.75</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>383.1</v>
+        <v>1168</v>
       </c>
       <c r="C38" t="n">
-        <v>39.04</v>
+        <v>38.32</v>
       </c>
       <c r="D38" t="n">
-        <v>54.17</v>
+        <v>53.82</v>
       </c>
       <c r="E38" t="n">
-        <v>-18.22</v>
+        <v>-12.9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1307.7</v>
+        <v>287.8</v>
       </c>
       <c r="C39" t="n">
-        <v>39.04</v>
+        <v>38.38</v>
       </c>
       <c r="D39" t="n">
-        <v>51.56</v>
+        <v>46.23</v>
       </c>
       <c r="E39" t="n">
-        <v>-15.08</v>
+        <v>-25.88</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3693.4</v>
+        <v>287.8</v>
       </c>
       <c r="C40" t="n">
-        <v>39.29</v>
+        <v>38.38</v>
       </c>
       <c r="D40" t="n">
-        <v>49.73</v>
+        <v>46.23</v>
       </c>
       <c r="E40" t="n">
-        <v>-16.4</v>
+        <v>-25.88</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>HDFCAMC</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2308.1</v>
+        <v>9778</v>
       </c>
       <c r="C41" t="n">
-        <v>39.37</v>
+        <v>38.52</v>
       </c>
       <c r="D41" t="n">
-        <v>48.64</v>
+        <v>52.59</v>
       </c>
       <c r="E41" t="n">
-        <v>-20.46</v>
+        <v>-20.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CHOLAFIN</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1580</v>
+        <v>900.35</v>
       </c>
       <c r="C42" t="n">
-        <v>39.8</v>
+        <v>38.74</v>
       </c>
       <c r="D42" t="n">
-        <v>51.77</v>
+        <v>54.87</v>
       </c>
       <c r="E42" t="n">
-        <v>-18.56</v>
+        <v>-21.69</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>178</v>
+        <v>1016.7</v>
       </c>
       <c r="C43" t="n">
-        <v>39.96</v>
+        <v>38.97</v>
       </c>
       <c r="D43" t="n">
-        <v>52.04</v>
+        <v>49.82</v>
       </c>
       <c r="E43" t="n">
-        <v>-19.5</v>
+        <v>-21.11</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1734.7</v>
+      </c>
+      <c r="C44" t="n">
+        <v>39.04</v>
+      </c>
+      <c r="D44" t="n">
+        <v>46.34</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-20.3</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1684.6</v>
+      </c>
+      <c r="C45" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="D45" t="n">
+        <v>47.55</v>
+      </c>
+      <c r="E45" t="n">
+        <v>-20.15</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2890</v>
+      </c>
+      <c r="C46" t="n">
+        <v>39.66</v>
+      </c>
+      <c r="D46" t="n">
+        <v>53.51</v>
+      </c>
+      <c r="E46" t="n">
+        <v>-14.51</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>3703.3</v>
+      </c>
+      <c r="C47" t="n">
+        <v>39.81</v>
+      </c>
+      <c r="D47" t="n">
+        <v>49.92</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-16.18</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>959.1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>39.92</v>
+      </c>
+      <c r="D48" t="n">
+        <v>53.28</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-21.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSI screener report 2026-10-17 07:56 UTC
</commit_message>
<xml_diff>
--- a/docs/nifty500_rsi_report.xlsx
+++ b/docs/nifty500_rsi_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -466,134 +466,134 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IRFC</t>
+          <t>AMBUJACEM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74.7</v>
+        <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>22.13</v>
+        <v>27.58</v>
       </c>
       <c r="D2" t="n">
-        <v>36.34</v>
+        <v>32.77</v>
       </c>
       <c r="E2" t="n">
-        <v>-44.1</v>
+        <v>-37.63</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMBUJACEM</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>351.5</v>
+        <v>11445</v>
       </c>
       <c r="C3" t="n">
-        <v>22.79</v>
+        <v>30.48</v>
       </c>
       <c r="D3" t="n">
-        <v>32.03</v>
+        <v>42.5</v>
       </c>
       <c r="E3" t="n">
-        <v>-39.1</v>
+        <v>-33.81</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>955</v>
+        <v>250.45</v>
       </c>
       <c r="C4" t="n">
-        <v>26.62</v>
+        <v>31.73</v>
       </c>
       <c r="D4" t="n">
-        <v>42.71</v>
+        <v>43.09</v>
       </c>
       <c r="E4" t="n">
-        <v>-24.86</v>
+        <v>-21.95</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>DMART</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1856.7</v>
+        <v>3342</v>
       </c>
       <c r="C5" t="n">
-        <v>27.16</v>
+        <v>32.28</v>
       </c>
       <c r="D5" t="n">
-        <v>35.27</v>
+        <v>40.94</v>
       </c>
       <c r="E5" t="n">
-        <v>-28.69</v>
+        <v>-27.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11420</v>
+        <v>4850</v>
       </c>
       <c r="C6" t="n">
-        <v>30.08</v>
+        <v>32.31</v>
       </c>
       <c r="D6" t="n">
-        <v>42.4</v>
+        <v>42.69</v>
       </c>
       <c r="E6" t="n">
-        <v>-33.96</v>
+        <v>-21.58</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>279.9</v>
+        <v>4850</v>
       </c>
       <c r="C7" t="n">
-        <v>30.11</v>
+        <v>32.31</v>
       </c>
       <c r="D7" t="n">
-        <v>33.24</v>
+        <v>42.69</v>
       </c>
       <c r="E7" t="n">
-        <v>-58.9</v>
+        <v>-21.58</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>249.15</v>
+        <v>1893.8</v>
       </c>
       <c r="C8" t="n">
-        <v>30.47</v>
+        <v>32.37</v>
       </c>
       <c r="D8" t="n">
-        <v>42.81</v>
+        <v>36.47</v>
       </c>
       <c r="E8" t="n">
-        <v>-22.36</v>
+        <v>-27.27</v>
       </c>
     </row>
     <row r="9">
@@ -603,757 +603,548 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>312</v>
+        <v>315.15</v>
       </c>
       <c r="C9" t="n">
-        <v>30.51</v>
+        <v>33.08</v>
       </c>
       <c r="D9" t="n">
-        <v>43.9</v>
+        <v>44.55</v>
       </c>
       <c r="E9" t="n">
-        <v>-23.94</v>
+        <v>-23.17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>162.57</v>
+        <v>869.4</v>
       </c>
       <c r="C10" t="n">
-        <v>30.58</v>
+        <v>33.35</v>
       </c>
       <c r="D10" t="n">
-        <v>35.36</v>
+        <v>38.78</v>
       </c>
       <c r="E10" t="n">
-        <v>-40.38</v>
+        <v>-30.67</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4825</v>
+        <v>246.1</v>
       </c>
       <c r="C11" t="n">
-        <v>30.89</v>
+        <v>33.4</v>
       </c>
       <c r="D11" t="n">
-        <v>42.3</v>
+        <v>38.8</v>
       </c>
       <c r="E11" t="n">
-        <v>-21.99</v>
+        <v>-68.75</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4825</v>
+        <v>286.85</v>
       </c>
       <c r="C12" t="n">
-        <v>30.89</v>
+        <v>33.5</v>
       </c>
       <c r="D12" t="n">
-        <v>42.3</v>
+        <v>33.77</v>
       </c>
       <c r="E12" t="n">
-        <v>-21.99</v>
+        <v>-31.21</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>860.5</v>
+        <v>978.9</v>
       </c>
       <c r="C13" t="n">
-        <v>31.55</v>
+        <v>33.58</v>
       </c>
       <c r="D13" t="n">
-        <v>38.23</v>
+        <v>44.51</v>
       </c>
       <c r="E13" t="n">
-        <v>-31.38</v>
+        <v>-22.98</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>MUTHOOTFIN</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>327.8</v>
+        <v>2598.3</v>
       </c>
       <c r="C14" t="n">
-        <v>31.63</v>
+        <v>33.66</v>
       </c>
       <c r="D14" t="n">
-        <v>42.65</v>
+        <v>47.16</v>
       </c>
       <c r="E14" t="n">
-        <v>-31.91</v>
+        <v>-36.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22080</v>
+        <v>2331.9</v>
       </c>
       <c r="C15" t="n">
-        <v>31.92</v>
+        <v>33.81</v>
       </c>
       <c r="D15" t="n">
-        <v>37.22</v>
+        <v>44.15</v>
       </c>
       <c r="E15" t="n">
-        <v>-26.42</v>
+        <v>-21.45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MAZDOCK</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2010</v>
+        <v>333.25</v>
       </c>
       <c r="C16" t="n">
-        <v>32.11</v>
+        <v>34.05</v>
       </c>
       <c r="D16" t="n">
-        <v>45.6</v>
+        <v>43.46</v>
       </c>
       <c r="E16" t="n">
-        <v>-30.42</v>
+        <v>-30.77</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1170.3</v>
+        <v>222</v>
       </c>
       <c r="C17" t="n">
-        <v>32.14</v>
+        <v>34.28</v>
       </c>
       <c r="D17" t="n">
-        <v>39.35</v>
+        <v>43.68</v>
       </c>
       <c r="E17" t="n">
-        <v>-26.5</v>
+        <v>-26.34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2796.2</v>
+        <v>22315</v>
       </c>
       <c r="C18" t="n">
-        <v>33.14</v>
+        <v>34.3</v>
       </c>
       <c r="D18" t="n">
-        <v>46.33</v>
+        <v>37.8</v>
       </c>
       <c r="E18" t="n">
-        <v>-26.46</v>
+        <v>-25.64</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>IRFC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>221.27</v>
+        <v>80.25</v>
       </c>
       <c r="C19" t="n">
-        <v>33.6</v>
+        <v>35.11</v>
       </c>
       <c r="D19" t="n">
-        <v>43.51</v>
+        <v>38.31</v>
       </c>
       <c r="E19" t="n">
-        <v>-26.59</v>
+        <v>-39.95</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2339.1</v>
+        <v>230.4</v>
       </c>
       <c r="C20" t="n">
-        <v>34.18</v>
+        <v>35.29</v>
       </c>
       <c r="D20" t="n">
-        <v>44.29</v>
+        <v>45.06</v>
       </c>
       <c r="E20" t="n">
-        <v>-21.2</v>
+        <v>-28.99</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>126.35</v>
+        <v>4608</v>
       </c>
       <c r="C21" t="n">
-        <v>34.22</v>
+        <v>35.47</v>
       </c>
       <c r="D21" t="n">
-        <v>43.45</v>
+        <v>55.32</v>
       </c>
       <c r="E21" t="n">
-        <v>-32.6</v>
+        <v>-23.55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>707.25</v>
+        <v>1265.5</v>
       </c>
       <c r="C22" t="n">
-        <v>34.32</v>
+        <v>36.35</v>
       </c>
       <c r="D22" t="n">
-        <v>37.19</v>
+        <v>49.35</v>
       </c>
       <c r="E22" t="n">
-        <v>-29.94</v>
+        <v>-17.82</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MUTHOOTFIN</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2624.7</v>
+        <v>263.5</v>
       </c>
       <c r="C23" t="n">
-        <v>34.35</v>
+        <v>36.71</v>
       </c>
       <c r="D23" t="n">
-        <v>47.66</v>
+        <v>30.8</v>
       </c>
       <c r="E23" t="n">
-        <v>-35.85</v>
+        <v>-37.5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>368.15</v>
+        <v>118.29</v>
       </c>
       <c r="C24" t="n">
-        <v>34.58</v>
+        <v>36.89</v>
       </c>
       <c r="D24" t="n">
-        <v>51.66</v>
+        <v>49.91</v>
       </c>
       <c r="E24" t="n">
-        <v>-21.41</v>
+        <v>-25.57</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>MAZDOCK</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>264</v>
+        <v>2092</v>
       </c>
       <c r="C25" t="n">
-        <v>35.72</v>
+        <v>37</v>
       </c>
       <c r="D25" t="n">
-        <v>39.93</v>
+        <v>46.87</v>
       </c>
       <c r="E25" t="n">
-        <v>-66.48</v>
+        <v>-26.28</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>300</v>
+        <v>3627.1</v>
       </c>
       <c r="C26" t="n">
-        <v>35.82</v>
+        <v>37.17</v>
       </c>
       <c r="D26" t="n">
-        <v>41.14</v>
+        <v>48.5</v>
       </c>
       <c r="E26" t="n">
-        <v>-22.19</v>
+        <v>-17.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>342.15</v>
+        <v>1656.8</v>
       </c>
       <c r="C27" t="n">
-        <v>36.01</v>
+        <v>37.36</v>
       </c>
       <c r="D27" t="n">
-        <v>44.37</v>
+        <v>46.32</v>
       </c>
       <c r="E27" t="n">
-        <v>-25.91</v>
+        <v>-21.46</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DMART</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3516.8</v>
+        <v>1729</v>
       </c>
       <c r="C28" t="n">
-        <v>36.03</v>
+        <v>38.68</v>
       </c>
       <c r="D28" t="n">
-        <v>42.84</v>
+        <v>46.13</v>
       </c>
       <c r="E28" t="n">
-        <v>-24.02</v>
+        <v>-20.56</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>10675</v>
+        <v>7890</v>
       </c>
       <c r="C29" t="n">
-        <v>36.33</v>
+        <v>38.92</v>
       </c>
       <c r="D29" t="n">
-        <v>46.14</v>
+        <v>55.29</v>
       </c>
       <c r="E29" t="n">
-        <v>-18.21</v>
+        <v>-13</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>173.8</v>
+        <v>376.85</v>
       </c>
       <c r="C30" t="n">
-        <v>37.22</v>
+        <v>38.95</v>
       </c>
       <c r="D30" t="n">
-        <v>50.49</v>
+        <v>53.09</v>
       </c>
       <c r="E30" t="n">
-        <v>-21.4</v>
+        <v>-19.55</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1301</v>
+        <v>175.5</v>
       </c>
       <c r="C31" t="n">
-        <v>37.63</v>
+        <v>39.04</v>
       </c>
       <c r="D31" t="n">
-        <v>43.87</v>
+        <v>51.11</v>
       </c>
       <c r="E31" t="n">
-        <v>-21.8</v>
+        <v>-20.63</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HDFCAMC</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2262.5</v>
+        <v>1211.2</v>
       </c>
       <c r="C32" t="n">
-        <v>37.82</v>
+        <v>39.06</v>
       </c>
       <c r="D32" t="n">
-        <v>47.37</v>
+        <v>41.92</v>
       </c>
       <c r="E32" t="n">
-        <v>-22.03</v>
+        <v>-23.93</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>266</v>
+        <v>2885.9</v>
       </c>
       <c r="C33" t="n">
-        <v>37.84</v>
+        <v>39.49</v>
       </c>
       <c r="D33" t="n">
-        <v>31.56</v>
+        <v>53.41</v>
       </c>
       <c r="E33" t="n">
-        <v>-36.91</v>
+        <v>-14.63</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>CHOLAFIN</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>861.65</v>
+        <v>1574.4</v>
       </c>
       <c r="C34" t="n">
-        <v>38.04</v>
+        <v>39.65</v>
       </c>
       <c r="D34" t="n">
-        <v>44.47</v>
+        <v>51.58</v>
       </c>
       <c r="E34" t="n">
-        <v>-19.42</v>
+        <v>-18.85</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>235.8</v>
+        <v>307.8</v>
       </c>
       <c r="C35" t="n">
-        <v>38.08</v>
+        <v>39.65</v>
       </c>
       <c r="D35" t="n">
-        <v>46.54</v>
+        <v>42.4</v>
       </c>
       <c r="E35" t="n">
-        <v>-27.32</v>
+        <v>-20.17</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>IOC</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1023.4</v>
+        <v>130.38</v>
       </c>
       <c r="C36" t="n">
-        <v>38.1</v>
+        <v>39.79</v>
       </c>
       <c r="D36" t="n">
-        <v>34.81</v>
+        <v>44.93</v>
       </c>
       <c r="E36" t="n">
-        <v>-39.44</v>
+        <v>-30.45</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>119.59</v>
+        <v>2920.9</v>
       </c>
       <c r="C37" t="n">
-        <v>38.16</v>
+        <v>39.95</v>
       </c>
       <c r="D37" t="n">
-        <v>50.54</v>
+        <v>48.94</v>
       </c>
       <c r="E37" t="n">
-        <v>-24.75</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>JSWSTEEL</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1168</v>
-      </c>
-      <c r="C38" t="n">
-        <v>38.32</v>
-      </c>
-      <c r="D38" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="E38" t="n">
-        <v>-12.9</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>BPCL</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>287.8</v>
-      </c>
-      <c r="C39" t="n">
-        <v>38.38</v>
-      </c>
-      <c r="D39" t="n">
-        <v>46.23</v>
-      </c>
-      <c r="E39" t="n">
-        <v>-25.88</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>BPCL</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>287.8</v>
-      </c>
-      <c r="C40" t="n">
-        <v>38.38</v>
-      </c>
-      <c r="D40" t="n">
-        <v>46.23</v>
-      </c>
-      <c r="E40" t="n">
-        <v>-25.88</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>BAJAJ-AUTO</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>9778</v>
-      </c>
-      <c r="C41" t="n">
-        <v>38.52</v>
-      </c>
-      <c r="D41" t="n">
-        <v>52.59</v>
-      </c>
-      <c r="E41" t="n">
-        <v>-20.9</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>HINDALCO</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>900.35</v>
-      </c>
-      <c r="C42" t="n">
-        <v>38.74</v>
-      </c>
-      <c r="D42" t="n">
-        <v>54.87</v>
-      </c>
-      <c r="E42" t="n">
-        <v>-21.69</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>JINDALSTEL</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1016.7</v>
-      </c>
-      <c r="C43" t="n">
-        <v>38.97</v>
-      </c>
-      <c r="D43" t="n">
-        <v>49.82</v>
-      </c>
-      <c r="E43" t="n">
-        <v>-21.11</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>BAJAJFINSV</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>1734.7</v>
-      </c>
-      <c r="C44" t="n">
-        <v>39.04</v>
-      </c>
-      <c r="D44" t="n">
-        <v>46.34</v>
-      </c>
-      <c r="E44" t="n">
-        <v>-20.3</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>SBILIFE</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>1684.6</v>
-      </c>
-      <c r="C45" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="D45" t="n">
-        <v>47.55</v>
-      </c>
-      <c r="E45" t="n">
-        <v>-20.15</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>GRASIM</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>2890</v>
-      </c>
-      <c r="C46" t="n">
-        <v>39.66</v>
-      </c>
-      <c r="D46" t="n">
-        <v>53.51</v>
-      </c>
-      <c r="E46" t="n">
-        <v>-14.51</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>3703.3</v>
-      </c>
-      <c r="C47" t="n">
-        <v>39.81</v>
-      </c>
-      <c r="D47" t="n">
-        <v>49.92</v>
-      </c>
-      <c r="E47" t="n">
-        <v>-16.18</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>959.1</v>
-      </c>
-      <c r="C48" t="n">
-        <v>39.92</v>
-      </c>
-      <c r="D48" t="n">
-        <v>53.28</v>
-      </c>
-      <c r="E48" t="n">
-        <v>-21.88</v>
+        <v>-23.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>